<commit_message>
mark attendance page divide
</commit_message>
<xml_diff>
--- a/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_Attendance.xlsx
+++ b/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_Attendance.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="74">
   <si>
     <t>Watumull Institute of Electronics Engineering &amp; Computer Technology</t>
   </si>
@@ -37,6 +37,9 @@
     <t>2026-07-21</t>
   </si>
   <si>
+    <t>2026-07-28</t>
+  </si>
+  <si>
     <t>Total Present</t>
   </si>
   <si>
@@ -49,7 +52,7 @@
     <t>ADSULE ANANYA ANIL</t>
   </si>
   <si>
-    <t>0.00%</t>
+    <t>50.00%</t>
   </si>
   <si>
     <t>ADURKAR JAYESH MAHESH</t>
@@ -661,14 +664,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -716,7 +719,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="20" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
@@ -735,33 +738,39 @@
       <c r="F6" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="7">
         <v>0</v>
       </c>
       <c r="D7" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="5">
         <v>1</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F7" s="5">
+        <v>1</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="7">
         <v>1</v>
@@ -770,18 +779,21 @@
         <v>1</v>
       </c>
       <c r="E8" s="5">
-        <v>0</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F8" s="5">
+        <v>0</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>3</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -790,38 +802,44 @@
         <v>1</v>
       </c>
       <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" s="7">
         <v>0</v>
       </c>
       <c r="D10" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="5">
+        <v>1</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>5</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" s="7">
         <v>1</v>
@@ -830,18 +848,21 @@
         <v>1</v>
       </c>
       <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>6</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C12" s="7">
         <v>1</v>
@@ -850,18 +871,21 @@
         <v>1</v>
       </c>
       <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" s="7">
         <v>1</v>
@@ -870,18 +894,21 @@
         <v>1</v>
       </c>
       <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F13" s="5">
+        <v>0</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="7">
         <v>1</v>
@@ -890,18 +917,21 @@
         <v>1</v>
       </c>
       <c r="E14" s="5">
-        <v>0</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="7">
         <v>1</v>
@@ -910,18 +940,21 @@
         <v>1</v>
       </c>
       <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C16" s="7">
         <v>1</v>
@@ -930,18 +963,21 @@
         <v>1</v>
       </c>
       <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17" s="7">
         <v>1</v>
@@ -950,18 +986,21 @@
         <v>1</v>
       </c>
       <c r="E17" s="5">
-        <v>0</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F17" s="5">
+        <v>0</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>12</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="7">
         <v>1</v>
@@ -970,18 +1009,21 @@
         <v>1</v>
       </c>
       <c r="E18" s="5">
-        <v>0</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6">
         <v>13</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -990,18 +1032,21 @@
         <v>1</v>
       </c>
       <c r="E19" s="5">
-        <v>0</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6">
         <v>14</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C20" s="7">
         <v>1</v>
@@ -1010,18 +1055,21 @@
         <v>1</v>
       </c>
       <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6">
         <v>15</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" s="7">
         <v>1</v>
@@ -1030,18 +1078,21 @@
         <v>1</v>
       </c>
       <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C22" s="7">
         <v>1</v>
@@ -1050,18 +1101,21 @@
         <v>1</v>
       </c>
       <c r="E22" s="5">
-        <v>0</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6">
         <v>17</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23" s="7">
         <v>1</v>
@@ -1070,18 +1124,21 @@
         <v>1</v>
       </c>
       <c r="E23" s="5">
-        <v>0</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>18</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C24" s="7">
         <v>1</v>
@@ -1090,18 +1147,21 @@
         <v>1</v>
       </c>
       <c r="E24" s="5">
-        <v>0</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="6">
         <v>19</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C25" s="7">
         <v>1</v>
@@ -1110,18 +1170,21 @@
         <v>1</v>
       </c>
       <c r="E25" s="5">
-        <v>0</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F25" s="5">
+        <v>0</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="6">
         <v>20</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C26" s="7">
         <v>1</v>
@@ -1130,18 +1193,21 @@
         <v>1</v>
       </c>
       <c r="E26" s="5">
-        <v>0</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="6">
         <v>21</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C27" s="7">
         <v>1</v>
@@ -1150,18 +1216,21 @@
         <v>1</v>
       </c>
       <c r="E27" s="5">
-        <v>0</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>22</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C28" s="7">
         <v>1</v>
@@ -1170,18 +1239,21 @@
         <v>1</v>
       </c>
       <c r="E28" s="5">
-        <v>0</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F28" s="5">
+        <v>0</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>23</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C29" s="7">
         <v>1</v>
@@ -1190,18 +1262,21 @@
         <v>1</v>
       </c>
       <c r="E29" s="5">
-        <v>0</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F29" s="5">
+        <v>0</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>24</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C30" s="7">
         <v>1</v>
@@ -1210,18 +1285,21 @@
         <v>1</v>
       </c>
       <c r="E30" s="5">
-        <v>0</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F30" s="5">
+        <v>0</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>25</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C31" s="7">
         <v>1</v>
@@ -1230,18 +1308,21 @@
         <v>1</v>
       </c>
       <c r="E31" s="5">
-        <v>0</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F31" s="5">
+        <v>0</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>26</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C32" s="7">
         <v>1</v>
@@ -1250,18 +1331,21 @@
         <v>1</v>
       </c>
       <c r="E32" s="5">
-        <v>0</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>27</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C33" s="7">
         <v>1</v>
@@ -1270,18 +1354,21 @@
         <v>1</v>
       </c>
       <c r="E33" s="5">
-        <v>0</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>28</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C34" s="7">
         <v>1</v>
@@ -1290,18 +1377,21 @@
         <v>1</v>
       </c>
       <c r="E34" s="5">
-        <v>0</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F34" s="5">
+        <v>0</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>29</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C35" s="7">
         <v>1</v>
@@ -1310,18 +1400,21 @@
         <v>1</v>
       </c>
       <c r="E35" s="5">
-        <v>0</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F35" s="5">
+        <v>0</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>30</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C36" s="7">
         <v>1</v>
@@ -1330,18 +1423,21 @@
         <v>1</v>
       </c>
       <c r="E36" s="5">
-        <v>0</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F36" s="5">
+        <v>0</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>31</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C37" s="7">
         <v>1</v>
@@ -1350,38 +1446,44 @@
         <v>1</v>
       </c>
       <c r="E37" s="5">
-        <v>0</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F37" s="5">
+        <v>0</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>32</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C38" s="7">
         <v>1</v>
       </c>
       <c r="D38" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E38" s="5">
-        <v>0</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F38" s="5">
+        <v>1</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>33</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C39" s="7">
         <v>1</v>
@@ -1390,18 +1492,21 @@
         <v>1</v>
       </c>
       <c r="E39" s="5">
-        <v>0</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F39" s="5">
+        <v>0</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="6">
         <v>34</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C40" s="7">
         <v>1</v>
@@ -1410,18 +1515,21 @@
         <v>1</v>
       </c>
       <c r="E40" s="5">
-        <v>0</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F40" s="5">
+        <v>0</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>35</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C41" s="7">
         <v>1</v>
@@ -1430,18 +1538,21 @@
         <v>1</v>
       </c>
       <c r="E41" s="5">
-        <v>0</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
         <v>36</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C42" s="7">
         <v>1</v>
@@ -1450,18 +1561,21 @@
         <v>1</v>
       </c>
       <c r="E42" s="5">
-        <v>0</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F42" s="5">
+        <v>0</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="6">
         <v>37</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C43" s="7">
         <v>1</v>
@@ -1470,18 +1584,21 @@
         <v>1</v>
       </c>
       <c r="E43" s="5">
-        <v>0</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F43" s="5">
+        <v>0</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
         <v>38</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C44" s="7">
         <v>1</v>
@@ -1490,18 +1607,21 @@
         <v>1</v>
       </c>
       <c r="E44" s="5">
-        <v>0</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F44" s="5">
+        <v>0</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>39</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C45" s="7">
         <v>1</v>
@@ -1510,18 +1630,21 @@
         <v>1</v>
       </c>
       <c r="E45" s="5">
-        <v>0</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F45" s="5">
+        <v>0</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
         <v>40</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C46" s="7">
         <v>1</v>
@@ -1530,18 +1653,21 @@
         <v>1</v>
       </c>
       <c r="E46" s="5">
-        <v>0</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F46" s="5">
+        <v>0</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="6">
         <v>41</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C47" s="7">
         <v>1</v>
@@ -1550,18 +1676,21 @@
         <v>1</v>
       </c>
       <c r="E47" s="5">
-        <v>0</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F47" s="5">
+        <v>0</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="6">
         <v>42</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C48" s="7">
         <v>1</v>
@@ -1570,18 +1699,21 @@
         <v>1</v>
       </c>
       <c r="E48" s="5">
-        <v>0</v>
-      </c>
-      <c r="F48" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F48" s="5">
+        <v>0</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>43</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C49" s="7">
         <v>1</v>
@@ -1590,18 +1722,21 @@
         <v>1</v>
       </c>
       <c r="E49" s="5">
-        <v>0</v>
-      </c>
-      <c r="F49" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F49" s="5">
+        <v>0</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>44</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C50" s="7">
         <v>1</v>
@@ -1610,18 +1745,21 @@
         <v>1</v>
       </c>
       <c r="E50" s="5">
-        <v>0</v>
-      </c>
-      <c r="F50" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F50" s="5">
+        <v>0</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="6">
         <v>45</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C51" s="7">
         <v>1</v>
@@ -1630,18 +1768,21 @@
         <v>1</v>
       </c>
       <c r="E51" s="5">
-        <v>0</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F51" s="5">
+        <v>0</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="6">
         <v>46</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C52" s="7">
         <v>1</v>
@@ -1650,18 +1791,21 @@
         <v>1</v>
       </c>
       <c r="E52" s="5">
-        <v>0</v>
-      </c>
-      <c r="F52" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="6">
         <v>47</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C53" s="7">
         <v>1</v>
@@ -1670,18 +1814,21 @@
         <v>1</v>
       </c>
       <c r="E53" s="5">
-        <v>0</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F53" s="5">
+        <v>0</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="6">
         <v>48</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C54" s="7">
         <v>1</v>
@@ -1690,18 +1837,21 @@
         <v>1</v>
       </c>
       <c r="E54" s="5">
-        <v>0</v>
-      </c>
-      <c r="F54" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F54" s="5">
+        <v>0</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="6">
         <v>49</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C55" s="7">
         <v>1</v>
@@ -1710,18 +1860,21 @@
         <v>1</v>
       </c>
       <c r="E55" s="5">
-        <v>0</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F55" s="5">
+        <v>0</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="6">
         <v>50</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C56" s="7">
         <v>1</v>
@@ -1730,18 +1883,21 @@
         <v>1</v>
       </c>
       <c r="E56" s="5">
-        <v>0</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F56" s="5">
+        <v>0</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="6">
         <v>51</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C57" s="7">
         <v>1</v>
@@ -1750,18 +1906,21 @@
         <v>1</v>
       </c>
       <c r="E57" s="5">
-        <v>0</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F57" s="5">
+        <v>0</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="6">
         <v>52</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C58" s="7">
         <v>1</v>
@@ -1770,18 +1929,21 @@
         <v>1</v>
       </c>
       <c r="E58" s="5">
-        <v>0</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F58" s="5">
+        <v>0</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="6">
         <v>53</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C59" s="7">
         <v>1</v>
@@ -1790,18 +1952,21 @@
         <v>1</v>
       </c>
       <c r="E59" s="5">
-        <v>0</v>
-      </c>
-      <c r="F59" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F59" s="5">
+        <v>0</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="6">
         <v>54</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C60" s="7">
         <v>1</v>
@@ -1810,18 +1975,21 @@
         <v>1</v>
       </c>
       <c r="E60" s="5">
-        <v>0</v>
-      </c>
-      <c r="F60" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F60" s="5">
+        <v>0</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="6">
         <v>55</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C61" s="7">
         <v>1</v>
@@ -1830,18 +1998,21 @@
         <v>1</v>
       </c>
       <c r="E61" s="5">
-        <v>0</v>
-      </c>
-      <c r="F61" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F61" s="5">
+        <v>0</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="6">
         <v>56</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C62" s="7">
         <v>1</v>
@@ -1850,18 +2021,21 @@
         <v>1</v>
       </c>
       <c r="E62" s="5">
-        <v>0</v>
-      </c>
-      <c r="F62" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F62" s="5">
+        <v>0</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="6">
         <v>57</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C63" s="7">
         <v>1</v>
@@ -1870,18 +2044,21 @@
         <v>1</v>
       </c>
       <c r="E63" s="5">
-        <v>0</v>
-      </c>
-      <c r="F63" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F63" s="5">
+        <v>0</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="6">
         <v>58</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C64" s="7">
         <v>1</v>
@@ -1890,18 +2067,21 @@
         <v>1</v>
       </c>
       <c r="E64" s="5">
-        <v>0</v>
-      </c>
-      <c r="F64" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F64" s="5">
+        <v>0</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="6">
         <v>59</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C65" s="7">
         <v>1</v>
@@ -1910,18 +2090,21 @@
         <v>1</v>
       </c>
       <c r="E65" s="5">
-        <v>0</v>
-      </c>
-      <c r="F65" s="9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F65" s="5">
+        <v>0</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="6">
         <v>60</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C66" s="7">
         <v>1</v>
@@ -1930,10 +2113,13 @@
         <v>1</v>
       </c>
       <c r="E66" s="5">
-        <v>0</v>
-      </c>
-      <c r="F66" s="9" t="s">
-        <v>14</v>
+        <v>2</v>
+      </c>
+      <c r="F66" s="5">
+        <v>0</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1944,6 +2130,6 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
whatsapp report is updated
</commit_message>
<xml_diff>
--- a/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_Attendance.xlsx
+++ b/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_Attendance.xlsx
@@ -918,16 +918,16 @@
         <v>1</v>
       </c>
       <c r="E13" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1672,16 +1672,16 @@
         <v>1</v>
       </c>
       <c r="E42" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G42" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1698,16 +1698,16 @@
         <v>1</v>
       </c>
       <c r="E43" s="5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G43" s="5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>